<commit_message>
Included more box save methods for keeping Box crystal_screens json updated
</commit_message>
<xml_diff>
--- a/Crystal_Sendoff_Sheet.xlsx
+++ b/Crystal_Sendoff_Sheet.xlsx
@@ -1,37 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29022"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_6A35D55597615CB44BF6E6D05A0500B0476EC48E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48AB7671-4B77-4489-B0B3-42DE37315F73}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_605DF7549771D48293B6E1D05A0500B0476EE42B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="135" windowWidth="21075" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Crystal_Sendoff_Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Vial</t>
   </si>
@@ -64,6 +53,25 @@
   </si>
   <si>
     <t>Port</t>
+  </si>
+  <si>
+    <t>1TEL_DARPin_Crystal Screen_A1_top_left_07-01-2025_07-01-2025_harvested</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Miles Bradford</t>
+  </si>
+  <si>
+    <t>07-01-2025, 07-01-2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Just a test
+</t>
   </si>
 </sst>
 </file>
@@ -482,14 +490,30 @@
       <c r="A2" s="1">
         <v>2</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
+      <c r="B2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="4">
+        <v>560</v>
+      </c>
+      <c r="F2" s="4">
+        <v>745</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
     </row>

</xml_diff>